<commit_message>
Make tasks peer-to-peer: anyone proposes, team reviews
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R99edeBGk6ca9TxhUj954w
</commit_message>
<xml_diff>
--- a/growth/Трекер_команды.xlsx
+++ b/growth/Трекер_команды.xlsx
@@ -124,7 +124,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Подкаст / видео / книга — заметки отправлены</t>
+          <t xml:space="preserve">Подкаст / видео / книга — заметки скинул в общий чат</t>
         </r>
       </text>
     </comment>
@@ -290,7 +290,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Подкаст / видео / книга — заметки отправлены</t>
+          <t xml:space="preserve">Подкаст / видео / книга — заметки скинул в общий чат</t>
         </r>
       </text>
     </comment>
@@ -456,7 +456,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Подкаст / видео / книга — заметки отправлены</t>
+          <t xml:space="preserve">Подкаст / видео / книга — заметки скинул в общий чат</t>
         </r>
       </text>
     </comment>
@@ -622,7 +622,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Подкаст / видео / книга — заметки отправлены</t>
+          <t xml:space="preserve">Подкаст / видео / книга — заметки скинул в общий чат</t>
         </r>
       </text>
     </comment>
@@ -788,7 +788,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Подкаст / видео / книга — заметки отправлены</t>
+          <t xml:space="preserve">Подкаст / видео / книга — заметки скинул в общий чат</t>
         </r>
       </text>
     </comment>
@@ -917,7 +917,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="895" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="282">
   <si>
     <t xml:space="preserve">🧱 НАША СИСТЕМА — команда</t>
   </si>
@@ -943,7 +943,7 @@
     <t xml:space="preserve">ЗАДАНИЯ</t>
   </si>
   <si>
-    <t xml:space="preserve">Лист «Задания»: что задал Бектур. Сделал → заметки по шаблону и скрин Бектуру. Шаблон: 1) Название и кто говорит  2) 3–5 главных мыслей своими словами  3) Цитата, которая зацепила  4) Что применю завтра  5) Вопрос / с чем не согласен</t>
+    <t xml:space="preserve">Лист «Задания»: задание может предложить любой из нас. Сделал → заметки по шаблону и скрин в общий чат, остальные дают отзыв. Все равны — нет главного и подчинённых. Шаблон: 1) Название и кто говорит  2) 3–5 главных мыслей своими словами  3) Цитата, которая зацепила  4) Что применю завтра  5) Вопрос / с чем не согласен</t>
   </si>
   <si>
     <t xml:space="preserve">КАЖДОЕ ВОСКРЕСЕНЬЕ</t>
@@ -1027,7 +1027,7 @@
     <t xml:space="preserve">Развитие 30–60 мин</t>
   </si>
   <si>
-    <t xml:space="preserve">Задание от Бектура</t>
+    <t xml:space="preserve">Общее задание</t>
   </si>
   <si>
     <t xml:space="preserve">Шахматы</t>
@@ -1297,10 +1297,13 @@
     <t xml:space="preserve">Познакомиться с 1 сильным человеком (учитель, предприниматель)</t>
   </si>
   <si>
-    <t xml:space="preserve">Задания от Бектура</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Бектур заполняет A–E и I–J, исполнитель — F–H и отправляет скрин заметок.</t>
+    <t xml:space="preserve">Общие задания</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Задание может предложить любой. Исполнитель заполняет G–I и кидает скрин заметок в общий чат, остальные пишут отзыв и оценку.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кто предложил</t>
   </si>
   <si>
     <t xml:space="preserve">Кому</t>
@@ -1324,19 +1327,25 @@
     <t xml:space="preserve">Сдал?</t>
   </si>
   <si>
-    <t xml:space="preserve">Отзыв Бектура</t>
+    <t xml:space="preserve">Отзыв команды</t>
   </si>
   <si>
     <t xml:space="preserve">Оценка 1–5</t>
   </si>
   <si>
+    <t xml:space="preserve">Бектур</t>
+  </si>
+  <si>
     <t xml:space="preserve">Юзер 2</t>
   </si>
   <si>
     <t xml:space="preserve">Посмотреть подкаст и выписать заметки по шаблону</t>
   </si>
   <si>
-    <t xml:space="preserve">ссылку скинет Бектур</t>
+    <t xml:space="preserve">ссылка в общем чате</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Команда</t>
   </si>
   <si>
     <t xml:space="preserve">Все</t>
@@ -1421,9 +1430,6 @@
   </si>
   <si>
     <t xml:space="preserve">Чему научился / ошибки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Бектур</t>
   </si>
   <si>
     <t xml:space="preserve">Подкаст</t>
@@ -2377,7 +2383,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
@@ -2474,7 +2480,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -2487,7 +2493,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -2500,63 +2506,63 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F5" s="25"/>
       <c r="G5" s="24" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="H5" s="24" t="n">
         <v>3</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
@@ -2569,7 +2575,7 @@
     </row>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="B7" s="12"/>
       <c r="C7" s="12"/>
@@ -2582,7 +2588,7 @@
     </row>
     <row r="8" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
@@ -2595,7 +2601,7 @@
     </row>
     <row r="9" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
@@ -2608,7 +2614,7 @@
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
@@ -2621,7 +2627,7 @@
     </row>
     <row r="11" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
@@ -2634,7 +2640,7 @@
     </row>
     <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
@@ -2647,7 +2653,7 @@
     </row>
     <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
@@ -2660,7 +2666,7 @@
     </row>
     <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
@@ -2673,7 +2679,7 @@
     </row>
     <row r="15" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
@@ -2686,7 +2692,7 @@
     </row>
     <row r="16" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
@@ -2699,7 +2705,7 @@
     </row>
     <row r="17" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
@@ -2712,7 +2718,7 @@
     </row>
     <row r="18" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
@@ -2725,7 +2731,7 @@
     </row>
     <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
@@ -2781,7 +2787,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -2791,7 +2797,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -2801,50 +2807,50 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -2853,10 +2859,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -2865,10 +2871,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="12"/>
@@ -2877,10 +2883,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
@@ -2889,10 +2895,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -2901,10 +2907,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -2913,10 +2919,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
@@ -2925,10 +2931,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
@@ -2937,10 +2943,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
@@ -2949,10 +2955,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
@@ -2961,10 +2967,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
@@ -2973,10 +2979,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
@@ -2985,10 +2991,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
@@ -2997,10 +3003,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
@@ -3009,10 +3015,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
@@ -3021,10 +3027,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
@@ -3033,10 +3039,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
@@ -3045,10 +3051,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
@@ -3057,10 +3063,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
@@ -3069,10 +3075,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
@@ -3081,10 +3087,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C26" s="12"/>
       <c r="D26" s="12"/>
@@ -3093,10 +3099,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12"/>
@@ -3105,10 +3111,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C28" s="12"/>
       <c r="D28" s="12"/>
@@ -3117,10 +3123,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C29" s="12"/>
       <c r="D29" s="12"/>
@@ -3129,10 +3135,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C30" s="12"/>
       <c r="D30" s="12"/>
@@ -3141,10 +3147,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C31" s="12"/>
       <c r="D31" s="12"/>
@@ -3153,10 +3159,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
@@ -3165,10 +3171,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
@@ -3177,10 +3183,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C34" s="12"/>
       <c r="D34" s="12"/>
@@ -3189,10 +3195,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C35" s="12"/>
       <c r="D35" s="12"/>
@@ -3201,10 +3207,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C36" s="12"/>
       <c r="D36" s="12"/>
@@ -3213,10 +3219,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C37" s="12"/>
       <c r="D37" s="12"/>
@@ -3225,10 +3231,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C38" s="12"/>
       <c r="D38" s="12"/>
@@ -3237,10 +3243,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C39" s="12"/>
       <c r="D39" s="12"/>
@@ -3249,10 +3255,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C40" s="12"/>
       <c r="D40" s="12"/>
@@ -3261,10 +3267,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C41" s="12"/>
       <c r="D41" s="12"/>
@@ -3273,10 +3279,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C42" s="12"/>
       <c r="D42" s="12"/>
@@ -3285,10 +3291,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C43" s="12"/>
       <c r="D43" s="12"/>
@@ -3297,10 +3303,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C44" s="12"/>
       <c r="D44" s="12"/>
@@ -3352,7 +3358,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -3367,7 +3373,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -3382,54 +3388,54 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
@@ -3440,19 +3446,19 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D6" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="E6" s="20" t="s">
         <v>203</v>
-      </c>
-      <c r="E6" s="20" t="s">
-        <v>201</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
@@ -3463,19 +3469,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
@@ -3486,19 +3492,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B8" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="C8" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="C8" s="20" t="s">
-        <v>205</v>
-      </c>
       <c r="D8" s="20" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
@@ -3509,19 +3515,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
@@ -3532,19 +3538,19 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
@@ -3555,19 +3561,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
@@ -3578,19 +3584,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
@@ -3601,19 +3607,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
@@ -3624,19 +3630,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
@@ -3647,19 +3653,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
@@ -3670,19 +3676,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
@@ -3693,19 +3699,19 @@
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E17" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
@@ -3716,19 +3722,19 @@
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B18" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="C18" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="C18" s="20" t="s">
-        <v>238</v>
-      </c>
       <c r="D18" s="20" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
@@ -3739,19 +3745,19 @@
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -3762,19 +3768,19 @@
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -3785,19 +3791,19 @@
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E21" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -3808,19 +3814,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E22" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
@@ -3831,19 +3837,19 @@
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E23" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -3854,19 +3860,19 @@
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E24" s="20" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -3877,19 +3883,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E25" s="20" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
@@ -3900,19 +3906,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C26" s="20" t="s">
+        <v>267</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>268</v>
+      </c>
+      <c r="E26" s="20" t="s">
         <v>265</v>
-      </c>
-      <c r="D26" s="20" t="s">
-        <v>266</v>
-      </c>
-      <c r="E26" s="20" t="s">
-        <v>263</v>
       </c>
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
@@ -3923,19 +3929,19 @@
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C27" s="20" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E27" s="20" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F27" s="12"/>
       <c r="G27" s="12"/>
@@ -3946,19 +3952,19 @@
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D28" s="20" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F28" s="12"/>
       <c r="G28" s="12"/>
@@ -3969,19 +3975,19 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C29" s="20" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D29" s="20" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E29" s="20" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F29" s="12"/>
       <c r="G29" s="12"/>
@@ -3992,19 +3998,19 @@
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C30" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="D30" s="20" t="s">
+        <v>281</v>
+      </c>
+      <c r="E30" s="20" t="s">
         <v>278</v>
-      </c>
-      <c r="D30" s="20" t="s">
-        <v>279</v>
-      </c>
-      <c r="E30" s="20" t="s">
-        <v>276</v>
       </c>
       <c r="F30" s="12"/>
       <c r="G30" s="12"/>
@@ -10240,13 +10246,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:Z67" type="list">
+      <formula1>"✅,❌"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="AA5:AB67" type="decimal">
       <formula1>0</formula1>
       <formula2>24</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:Z67" type="list">
-      <formula1>"✅,❌"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -13260,13 +13266,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="AA5:AB67" type="decimal">
+      <formula1>0</formula1>
+      <formula2>24</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:Z67" type="list">
       <formula1>"✅,❌"</formula1>
       <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="AA5:AB67" type="decimal">
-      <formula1>0</formula1>
-      <formula2>24</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -20627,18 +20633,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20654,6 +20662,7 @@
       <c r="H1" s="5"/>
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
@@ -20668,6 +20677,7 @@
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
       <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
@@ -20700,182 +20710,209 @@
       <c r="J4" s="15" t="s">
         <v>136</v>
       </c>
+      <c r="K4" s="15" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="n">
         <v>46325</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="E5" s="21" t="n">
+        <v>140</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="F5" s="21" t="n">
         <v>46325</v>
       </c>
-      <c r="F5" s="12"/>
       <c r="G5" s="12"/>
       <c r="H5" s="12"/>
       <c r="I5" s="12"/>
       <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="n">
         <v>46327</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="E6" s="21" t="n">
+        <v>144</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="F6" s="21" t="n">
         <v>46329</v>
       </c>
-      <c r="F6" s="12"/>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
       <c r="I6" s="12"/>
       <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="n">
         <v>46329</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>143</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="E7" s="21" t="n">
+        <v>146</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="F7" s="21" t="n">
         <v>46331</v>
       </c>
-      <c r="F7" s="12"/>
       <c r="G7" s="12"/>
       <c r="H7" s="12"/>
       <c r="I7" s="12"/>
       <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="n">
         <v>46331</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="E8" s="21" t="n">
+        <v>148</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="F8" s="21" t="n">
         <v>46333</v>
       </c>
-      <c r="F8" s="12"/>
       <c r="G8" s="12"/>
       <c r="H8" s="12"/>
       <c r="I8" s="12"/>
       <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="n">
         <v>46334</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="E9" s="21" t="n">
+        <v>150</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="F9" s="21" t="n">
         <v>46334</v>
       </c>
-      <c r="F9" s="12"/>
       <c r="G9" s="12"/>
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
       <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="n">
         <v>46336</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="E10" s="21" t="n">
+        <v>152</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F10" s="21" t="n">
         <v>46338</v>
       </c>
-      <c r="F10" s="12"/>
       <c r="G10" s="12"/>
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
       <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="n">
         <v>46338</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="E11" s="21" t="n">
+        <v>154</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="F11" s="21" t="n">
         <v>46340</v>
       </c>
-      <c r="F11" s="12"/>
       <c r="G11" s="12"/>
       <c r="H11" s="12"/>
       <c r="I11" s="12"/>
       <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="n">
         <v>46339</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="E12" s="21" t="n">
+        <v>156</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="F12" s="21" t="n">
         <v>46340</v>
       </c>
-      <c r="F12" s="12"/>
       <c r="G12" s="12"/>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
       <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
     </row>
     <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="12"/>
@@ -20888,6 +20925,7 @@
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
       <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="12"/>
@@ -20900,6 +20938,7 @@
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
       <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="12"/>
@@ -20912,6 +20951,7 @@
       <c r="H15" s="12"/>
       <c r="I15" s="12"/>
       <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="12"/>
@@ -20924,6 +20964,7 @@
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
       <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12"/>
@@ -20936,6 +20977,7 @@
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
       <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12"/>
@@ -20948,6 +20990,7 @@
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
       <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12"/>
@@ -20960,6 +21003,7 @@
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
       <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12"/>
@@ -20972,6 +21016,7 @@
       <c r="H20" s="12"/>
       <c r="I20" s="12"/>
       <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12"/>
@@ -20984,6 +21029,7 @@
       <c r="H21" s="12"/>
       <c r="I21" s="12"/>
       <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12"/>
@@ -20996,6 +21042,7 @@
       <c r="H22" s="12"/>
       <c r="I22" s="12"/>
       <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12"/>
@@ -21008,6 +21055,7 @@
       <c r="H23" s="12"/>
       <c r="I23" s="12"/>
       <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="12"/>
@@ -21020,6 +21068,7 @@
       <c r="H24" s="12"/>
       <c r="I24" s="12"/>
       <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12"/>
@@ -21032,6 +21081,7 @@
       <c r="H25" s="12"/>
       <c r="I25" s="12"/>
       <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
     </row>
     <row r="26" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="12"/>
@@ -21044,6 +21094,7 @@
       <c r="H26" s="12"/>
       <c r="I26" s="12"/>
       <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
     </row>
     <row r="27" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="12"/>
@@ -21056,6 +21107,7 @@
       <c r="H27" s="12"/>
       <c r="I27" s="12"/>
       <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
     </row>
     <row r="28" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="12"/>
@@ -21068,6 +21120,7 @@
       <c r="H28" s="12"/>
       <c r="I28" s="12"/>
       <c r="J28" s="12"/>
+      <c r="K28" s="12"/>
     </row>
     <row r="29" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12"/>
@@ -21080,6 +21133,7 @@
       <c r="H29" s="12"/>
       <c r="I29" s="12"/>
       <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
     </row>
     <row r="30" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="12"/>
@@ -21092,6 +21146,7 @@
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
       <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="12"/>
@@ -21104,6 +21159,7 @@
       <c r="H31" s="12"/>
       <c r="I31" s="12"/>
       <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
     </row>
     <row r="32" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="12"/>
@@ -21116,6 +21172,7 @@
       <c r="H32" s="12"/>
       <c r="I32" s="12"/>
       <c r="J32" s="12"/>
+      <c r="K32" s="12"/>
     </row>
     <row r="33" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="12"/>
@@ -21128,6 +21185,7 @@
       <c r="H33" s="12"/>
       <c r="I33" s="12"/>
       <c r="J33" s="12"/>
+      <c r="K33" s="12"/>
     </row>
     <row r="34" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="12"/>
@@ -21140,6 +21198,7 @@
       <c r="H34" s="12"/>
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
     </row>
     <row r="35" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="12"/>
@@ -21152,6 +21211,7 @@
       <c r="H35" s="12"/>
       <c r="I35" s="12"/>
       <c r="J35" s="12"/>
+      <c r="K35" s="12"/>
     </row>
     <row r="36" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="12"/>
@@ -21164,6 +21224,7 @@
       <c r="H36" s="12"/>
       <c r="I36" s="12"/>
       <c r="J36" s="12"/>
+      <c r="K36" s="12"/>
     </row>
     <row r="37" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="12"/>
@@ -21176,6 +21237,7 @@
       <c r="H37" s="12"/>
       <c r="I37" s="12"/>
       <c r="J37" s="12"/>
+      <c r="K37" s="12"/>
     </row>
     <row r="38" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="12"/>
@@ -21188,6 +21250,7 @@
       <c r="H38" s="12"/>
       <c r="I38" s="12"/>
       <c r="J38" s="12"/>
+      <c r="K38" s="12"/>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="12"/>
@@ -21200,6 +21263,7 @@
       <c r="H39" s="12"/>
       <c r="I39" s="12"/>
       <c r="J39" s="12"/>
+      <c r="K39" s="12"/>
     </row>
     <row r="40" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="12"/>
@@ -21212,6 +21276,7 @@
       <c r="H40" s="12"/>
       <c r="I40" s="12"/>
       <c r="J40" s="12"/>
+      <c r="K40" s="12"/>
     </row>
     <row r="41" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="12"/>
@@ -21224,6 +21289,7 @@
       <c r="H41" s="12"/>
       <c r="I41" s="12"/>
       <c r="J41" s="12"/>
+      <c r="K41" s="12"/>
     </row>
     <row r="42" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="12"/>
@@ -21236,6 +21302,7 @@
       <c r="H42" s="12"/>
       <c r="I42" s="12"/>
       <c r="J42" s="12"/>
+      <c r="K42" s="12"/>
     </row>
     <row r="43" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="12"/>
@@ -21248,6 +21315,7 @@
       <c r="H43" s="12"/>
       <c r="I43" s="12"/>
       <c r="J43" s="12"/>
+      <c r="K43" s="12"/>
     </row>
     <row r="44" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="12"/>
@@ -21260,6 +21328,7 @@
       <c r="H44" s="12"/>
       <c r="I44" s="12"/>
       <c r="J44" s="12"/>
+      <c r="K44" s="12"/>
     </row>
     <row r="45" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="12"/>
@@ -21272,6 +21341,7 @@
       <c r="H45" s="12"/>
       <c r="I45" s="12"/>
       <c r="J45" s="12"/>
+      <c r="K45" s="12"/>
     </row>
     <row r="46" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="12"/>
@@ -21284,6 +21354,7 @@
       <c r="H46" s="12"/>
       <c r="I46" s="12"/>
       <c r="J46" s="12"/>
+      <c r="K46" s="12"/>
     </row>
     <row r="47" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="12"/>
@@ -21296,6 +21367,7 @@
       <c r="H47" s="12"/>
       <c r="I47" s="12"/>
       <c r="J47" s="12"/>
+      <c r="K47" s="12"/>
     </row>
     <row r="48" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="12"/>
@@ -21308,6 +21380,7 @@
       <c r="H48" s="12"/>
       <c r="I48" s="12"/>
       <c r="J48" s="12"/>
+      <c r="K48" s="12"/>
     </row>
     <row r="49" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="12"/>
@@ -21320,6 +21393,7 @@
       <c r="H49" s="12"/>
       <c r="I49" s="12"/>
       <c r="J49" s="12"/>
+      <c r="K49" s="12"/>
     </row>
     <row r="50" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="12"/>
@@ -21332,6 +21406,7 @@
       <c r="H50" s="12"/>
       <c r="I50" s="12"/>
       <c r="J50" s="12"/>
+      <c r="K50" s="12"/>
     </row>
     <row r="51" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="12"/>
@@ -21344,6 +21419,7 @@
       <c r="H51" s="12"/>
       <c r="I51" s="12"/>
       <c r="J51" s="12"/>
+      <c r="K51" s="12"/>
     </row>
     <row r="52" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="12"/>
@@ -21356,47 +21432,52 @@
       <c r="H52" s="12"/>
       <c r="I52" s="12"/>
       <c r="J52" s="12"/>
+      <c r="K52" s="12"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="22" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C54" s="0" t="str">
-        <f aca="false">COUNTIF(H5:H52,"✅")&amp;" из "&amp;COUNTA(C5:C52)</f>
+        <f aca="false">COUNTIF(I5:I52,"✅")&amp;" из "&amp;COUNTA(D5:D52)</f>
         <v>0 из 8</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="22" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C55" s="0" t="str">
-        <f aca="false">IFERROR(ROUND(AVERAGE(J5:J52),1),"—")</f>
+        <f aca="false">IFERROR(ROUND(AVERAGE(K5:K52),1),"—")</f>
         <v>—</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H52">
+  <conditionalFormatting sqref="I5:I52">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"✅"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B52" type="list">
+  <dataValidations count="4">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C52" type="list">
       <formula1>"Бектур,Юзер 1,Юзер 2,Юзер 3,Юзер 4,Все"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H52" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I52" type="list">
       <formula1>"✅,❌"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J52" type="whole">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K52" type="whole">
       <formula1>1</formula1>
       <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B52" type="list">
+      <formula1>"Бектур,Юзер 1,Юзер 2,Юзер 3,Юзер 4,Команда"</formula1>
+      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>